<commit_message>
class variables vs instance varibales
</commit_message>
<xml_diff>
--- a/topics.xlsx
+++ b/topics.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>OOP</t>
   </si>
@@ -46,6 +46,30 @@
   </si>
   <si>
     <t>Conclusion</t>
+  </si>
+  <si>
+    <t>getter &amp; setters</t>
+  </si>
+  <si>
+    <t>static &amp; class Method</t>
+  </si>
+  <si>
+    <t>Magic/Dunder Method</t>
+  </si>
+  <si>
+    <t>Exception Handling</t>
+  </si>
+  <si>
+    <t>Custom Exceptions</t>
+  </si>
+  <si>
+    <t>map,filter and reduce</t>
+  </si>
+  <si>
+    <t>walrus operator</t>
+  </si>
+  <si>
+    <t>Args &amp;kwargs</t>
   </si>
 </sst>
 </file>
@@ -405,7 +429,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -642,6 +666,15 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -689,7 +722,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -697,33 +730,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="11" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="12" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="13" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="14" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="15" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="25" borderId="16" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="11" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="12" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="13" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="14" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="15" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="25" borderId="16" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="45"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1046,10 +1088,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="E5:Y7"/>
+  <dimension ref="E5:Y15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="7" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6328125" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" customWidth="1"/>
     <col min="8" max="8" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="10" max="16" width="7.1796875" bestFit="1" customWidth="1"/>
@@ -1061,107 +1105,163 @@
   <sheetData>
     <row r="5" spans="5:25" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="5:25" ht="41.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>46205</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>46206</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="5">
         <v>46207</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>46208</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="5">
         <v>46209</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>46210</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="3">
         <v>46211</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="3">
         <v>46212</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="5">
         <v>46213</v>
       </c>
-      <c r="N6" s="4">
+      <c r="N6" s="3">
         <v>46214</v>
       </c>
-      <c r="O6" s="6">
+      <c r="O6" s="5">
         <v>46215</v>
       </c>
-      <c r="P6" s="7">
+      <c r="P6" s="6">
         <v>46216</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="Q6" s="3">
         <v>46217</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="4">
         <v>46218</v>
       </c>
-      <c r="S6" s="8">
+      <c r="S6" s="7">
         <v>46219</v>
       </c>
-      <c r="T6" s="9">
+      <c r="T6" s="8">
         <v>46220</v>
       </c>
-      <c r="U6" s="4">
+      <c r="U6" s="3">
         <v>46221</v>
       </c>
-      <c r="V6" s="4">
+      <c r="V6" s="3">
         <v>46222</v>
       </c>
-      <c r="W6" s="5">
+      <c r="W6" s="4">
         <v>46223</v>
       </c>
-      <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
+      <c r="X6" s="9"/>
+      <c r="Y6" s="9"/>
     </row>
     <row r="7" spans="5:25" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="3" t="s">
+      <c r="G7" s="11"/>
+      <c r="H7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2" t="s">
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2" t="s">
+      <c r="R7" s="11"/>
+      <c r="S7" s="11"/>
+      <c r="T7" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="U7" s="2"/>
-      <c r="V7" s="11"/>
-      <c r="W7" s="12" t="s">
+      <c r="U7" s="11"/>
+      <c r="V7" s="12"/>
+      <c r="W7" s="10" t="s">
         <v>8</v>
       </c>
+    </row>
+    <row r="8" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F8" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" s="15"/>
+    </row>
+    <row r="9" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F9" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="13"/>
+    </row>
+    <row r="10" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F11" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F13" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F14" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="14"/>
+    </row>
+    <row r="15" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="13">
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="J7:M7"/>
     <mergeCell ref="N7:P7"/>

</xml_diff>

<commit_message>
class method in OOP
</commit_message>
<xml_diff>
--- a/topics.xlsx
+++ b/topics.xlsx
@@ -722,7 +722,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -765,6 +765,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1088,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="E5:Y15"/>
+  <dimension ref="E5:Y16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="8.90625" bestFit="1" customWidth="1"/>
@@ -1211,57 +1214,61 @@
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F9" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="13"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
     </row>
     <row r="10" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F10" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G10" s="13"/>
     </row>
     <row r="11" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F11" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G11" s="13"/>
     </row>
     <row r="12" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F12" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G12" s="13"/>
     </row>
     <row r="13" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F13" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G13" s="13"/>
     </row>
     <row r="14" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F14" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="14"/>
+      <c r="F14" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="14"/>
+    </row>
+    <row r="16" spans="5:25" x14ac:dyDescent="0.35">
+      <c r="F16" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="13"/>
+      <c r="G16" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="F13:G13"/>
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="J7:M7"/>
     <mergeCell ref="N7:P7"/>

</xml_diff>

<commit_message>
magic / dunder methods in OOP classes
</commit_message>
<xml_diff>
--- a/topics.xlsx
+++ b/topics.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>OOP</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>Args &amp;kwargs</t>
+  </si>
+  <si>
+    <t>class variable vs instance</t>
   </si>
 </sst>
 </file>
@@ -722,7 +725,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -768,6 +771,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1096,7 +1102,7 @@
   <cols>
     <col min="5" max="5" width="8.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.6328125" customWidth="1"/>
-    <col min="7" max="7" width="9.7265625" customWidth="1"/>
+    <col min="7" max="7" width="13.1796875" customWidth="1"/>
     <col min="8" max="8" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="10" max="16" width="7.1796875" bestFit="1" customWidth="1"/>
@@ -1214,14 +1220,16 @@
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F9" s="16"/>
+      <c r="F9" s="16" t="s">
+        <v>17</v>
+      </c>
       <c r="G9" s="16"/>
     </row>
     <row r="10" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="13"/>
+      <c r="G10" s="17"/>
     </row>
     <row r="11" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F11" s="13" t="s">
@@ -1260,10 +1268,11 @@
       <c r="G16" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F9:G9"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="F11:G11"/>

</xml_diff>

<commit_message>
map reduce and filter functions
</commit_message>
<xml_diff>
--- a/topics.xlsx
+++ b/topics.xlsx
@@ -432,7 +432,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -678,6 +678,30 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -725,7 +749,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -767,14 +791,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1188,17 +1218,17 @@
       <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11" t="s">
+      <c r="K7" s="18"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="19"/>
       <c r="Q7" s="11" t="s">
         <v>6</v>
       </c>
@@ -1214,16 +1244,16 @@
       </c>
     </row>
     <row r="8" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="15"/>
+      <c r="G8" s="16"/>
     </row>
     <row r="9" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G9" s="16"/>
+      <c r="G9" s="15"/>
     </row>
     <row r="10" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F10" s="17" t="s">
@@ -1232,10 +1262,10 @@
       <c r="G10" s="17"/>
     </row>
     <row r="11" spans="5:25" x14ac:dyDescent="0.35">
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="17"/>
     </row>
     <row r="12" spans="5:25" x14ac:dyDescent="0.35">
       <c r="F12" s="13" t="s">
@@ -1279,10 +1309,10 @@
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="N7:P7"/>
     <mergeCell ref="Q7:S7"/>
     <mergeCell ref="T7:V7"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="M7:P7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>